<commit_message>
Actualizar datos: modelo y padrón del catastro (corrida diaria)
Regenerados por escanear + descargar_padron + cruce: modelo.json, pedimentos
(geojson/xlsx) y capas catastro_*.geojson.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out_2026/pedimentos.xlsx
+++ b/out_2026/pedimentos.xlsx
@@ -696,13 +696,13 @@
         <v>2968.97</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>-29.719982</v>
+        <v>-29.677908</v>
       </c>
       <c r="M5" t="n">
-        <v>-69.28144500000001</v>
+        <v>-69.273838</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1139,13 +1139,13 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>-28.98072</v>
+        <v>-28.985689</v>
       </c>
       <c r="M13" t="n">
-        <v>-69.032003</v>
+        <v>-69.011585</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -2638,13 +2638,13 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L42" t="n">
-        <v>-32.226455</v>
+        <v>-32.209647</v>
       </c>
       <c r="M42" t="n">
-        <v>-69.835066</v>
+        <v>-69.830049</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>

</xml_diff>